<commit_message>
Atualização automática portal mariana
</commit_message>
<xml_diff>
--- a/upload/contabancaria.xlsx
+++ b/upload/contabancaria.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J181"/>
+  <dimension ref="A1:J190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7641,17 +7641,377 @@
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="inlineStr"/>
-      <c r="B181" t="inlineStr"/>
-      <c r="C181" t="inlineStr"/>
-      <c r="D181" t="inlineStr"/>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
-      <c r="H181" t="inlineStr"/>
-      <c r="I181" t="inlineStr"/>
+      <c r="A181" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B181" t="n">
+        <v>8</v>
+      </c>
+      <c r="C181" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G181" t="n">
+        <v>9445683</v>
+      </c>
+      <c r="H181" t="n">
+        <v>80</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
       <c r="J181" t="n">
-        <v>367329713</v>
+        <v>2076547.8</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B182" t="n">
+        <v>8</v>
+      </c>
+      <c r="C182" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G182" t="n">
+        <v>9445684</v>
+      </c>
+      <c r="H182" t="n">
+        <v>80</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J182" t="n">
+        <v>39854.57</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B183" t="n">
+        <v>8</v>
+      </c>
+      <c r="C183" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G183" t="n">
+        <v>9445703</v>
+      </c>
+      <c r="H183" t="n">
+        <v>80</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J183" t="n">
+        <v>390802.66</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B184" t="n">
+        <v>8</v>
+      </c>
+      <c r="C184" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G184" t="n">
+        <v>9445716</v>
+      </c>
+      <c r="H184" t="n">
+        <v>80</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J184" t="n">
+        <v>10788294.8</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B185" t="n">
+        <v>8</v>
+      </c>
+      <c r="C185" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G185" t="n">
+        <v>9445718</v>
+      </c>
+      <c r="H185" t="n">
+        <v>80</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J185" t="n">
+        <v>2793637.88</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B186" t="n">
+        <v>8</v>
+      </c>
+      <c r="C186" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G186" t="n">
+        <v>9445719</v>
+      </c>
+      <c r="H186" t="n">
+        <v>80</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J186" t="n">
+        <v>4437363.18</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B187" t="n">
+        <v>8</v>
+      </c>
+      <c r="C187" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G187" t="n">
+        <v>9445721</v>
+      </c>
+      <c r="H187" t="n">
+        <v>80</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J187" t="n">
+        <v>3260698.08</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B188" t="n">
+        <v>8</v>
+      </c>
+      <c r="C188" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G188" t="n">
+        <v>9445763</v>
+      </c>
+      <c r="H188" t="n">
+        <v>80</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J188" t="n">
+        <v>1244405.03</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B189" t="n">
+        <v>8</v>
+      </c>
+      <c r="C189" t="n">
+        <v>9999</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>EMG - ADMINISTRACAO DIRETA</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>1321.01.0.1.01.000</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>REMUNERACAO DEPOSITOS BANCARIOS - PRINC.</t>
+        </is>
+      </c>
+      <c r="G189" t="n">
+        <v>9447774</v>
+      </c>
+      <c r="H189" t="n">
+        <v>80</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>RECURSOS DO ACORDO DE REPACTUACAO DO RIO DOCE</t>
+        </is>
+      </c>
+      <c r="J189" t="n">
+        <v>1506.26</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr"/>
+      <c r="B190" t="inlineStr"/>
+      <c r="C190" t="inlineStr"/>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="inlineStr"/>
+      <c r="J190" t="n">
+        <v>392362823.26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>